<commit_message>
feat: concluir requisito 5 e implementar navegação entre requisitos
</commit_message>
<xml_diff>
--- a/public/documents/requirement4/4_2/4_2_modelo_partes_interessadas.xlsx
+++ b/public/documents/requirement4/4_2/4_2_modelo_partes_interessadas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiff\integra-sgi\integra-sgi\src\assets\documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiff\integra-sgi\integra-sgi\public\documents\requirement4\4_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF02C1E-EBE1-487B-9864-73F699F74FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CBF52C5-737E-4170-AF40-1D555D9C6A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{0948FCCB-8106-4B64-891A-E538C6031D21}"/>
   </bookViews>
@@ -221,11 +221,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -641,12 +641,12 @@
     </row>
     <row r="2" spans="2:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="5"/>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="5"/>
@@ -679,7 +679,7 @@
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" ht="7.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="4"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
@@ -705,7 +705,7 @@
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -720,17 +720,18 @@
         <v>19</v>
       </c>
     </row>
+    <row r="15" spans="2:6" ht="5.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="2:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="7" t="s">
         <v>3</v>
       </c>
     </row>
@@ -821,7 +822,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
-    <oddFooter>&amp;L&amp;"Cambria,Normal"MODELO 4.2 -  Matriz das Partes Interessadas&amp;C&amp;"Cambria,Negrito"&amp;P &amp;"Cambria,Normal"de &amp;"Cambria,Negrito"&amp;N&amp;R&amp;"Cambria,Normal"R0 - data</oddFooter>
+    <oddFooter>&amp;L&amp;"Cambria,Normal"4.2 -  Matriz das Partes Interessadas&amp;C&amp;"Cambria,Negrito"&amp;P &amp;"Cambria,Normal"de &amp;"Cambria,Negrito"&amp;N&amp;R&amp;"Cambria,Normal"R0 - data</oddFooter>
   </headerFooter>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: adicionar novos modelos e guias de elaboração dos requisitos
</commit_message>
<xml_diff>
--- a/public/documents/requirement4/4_2/4_2_modelo_partes_interessadas.xlsx
+++ b/public/documents/requirement4/4_2/4_2_modelo_partes_interessadas.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiff\integra-sgi\integra-sgi\public\documents\requirement4\4_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CBF52C5-737E-4170-AF40-1D555D9C6A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7669CAFC-2D06-4C3D-86E7-5EB7730365C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{0948FCCB-8106-4B64-891A-E538C6031D21}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{0948FCCB-8106-4B64-891A-E538C6031D21}"/>
   </bookViews>
   <sheets>
-    <sheet name="Folha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Partes Interessadas" sheetId="1" r:id="rId1"/>
+    <sheet name="Explicação" sheetId="3" r:id="rId2"/>
+    <sheet name="Guia de Preenchimento" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,8 +40,73 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Thiffany Gabrielle</author>
+  </authors>
+  <commentList>
+    <comment ref="B4" authorId="0" shapeId="0" xr:uid="{87FE19B7-9018-474A-A53A-1A3E43101DD0}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Thiffany Gabrielle:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Verificar Explicações
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C12" authorId="0" shapeId="0" xr:uid="{BE1109FF-891E-43DD-8A4A-484E6D2B2887}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Thiffany Gabrielle:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+deve ser indicado é a frequência de revisão do documento.
+Por exemplo:
+anualmente
+sempre que necessário
+durante a Revisão pela Gestão
+a cada 12 meses
+sempre que houver alterações significativas</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="55">
   <si>
     <t>Parte Interessada</t>
   </si>
@@ -108,13 +175,135 @@
   </si>
   <si>
     <t xml:space="preserve">Esta informação é revista -------------------  e sempre que ocorram alterações relevantes no contexto da organização ou </t>
+  </si>
+  <si>
+    <t>Coluna</t>
+  </si>
+  <si>
+    <t>Como preencher</t>
+  </si>
+  <si>
+    <t>Exemplos</t>
+  </si>
+  <si>
+    <t>Identifique a pessoa, grupo ou entidade que pode influenciar ou ser influenciada pelas atividades da organização.</t>
+  </si>
+  <si>
+    <t>Clientes, Trabalhadores, Fornecedores, APA, ACT, Comunidade Local, Organismos de Certificação.</t>
+  </si>
+  <si>
+    <t>Produto de qualidade, entrega no prazo, ambiente de trabalho seguro, pagamentos atempados, cumprimento da legislação ambiental.</t>
+  </si>
+  <si>
+    <t>Pagamento dentro do prazo, cumprimento das regras de segurança, fornecimento de matéria-prima conforme especificação, colaboração em auditorias.</t>
+  </si>
+  <si>
+    <t>Indique a legislação, normas, contratos ou outros requisitos associados à relação com essa parte interessada. Quando não existirem requisitos específicos, pode indicar "Não aplicável".</t>
+  </si>
+  <si>
+    <t>ISO 9001, ISO 14001, ISO 45001, legislação laboral, legislação ambiental, contratos, regulamentos internos.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Registe aquilo que essa parte interessada espera receber da organização, quais são as suas necessidades, preocupações ou requisitos. Pergunte: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Cambria"/>
+        <family val="1"/>
+      </rPr>
+      <t>"O que esta parte interessada espera de nós?"</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Registe aquilo que a organização espera dessa parte interessada para garantir o bom funcionamento do SGI. Pergunte: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Cambria"/>
+        <family val="1"/>
+      </rPr>
+      <t>"O que precisamos desta parte interessada?"</t>
+    </r>
+  </si>
+  <si>
+    <t>Recomendações para o preenchimento</t>
+  </si>
+  <si>
+    <t>Considere apenas as partes interessadas que tenham influência significativa sobre a organização ou possam ser afetadas pelas suas atividades.</t>
+  </si>
+  <si>
+    <t>Utilize descrições objetivas e específicas, evitando textos demasiado longos.</t>
+  </si>
+  <si>
+    <t>Baseie as informações em evidências, contratos, legislação, reuniões, reclamações, questionários ou experiência operacional.</t>
+  </si>
+  <si>
+    <t>Sempre que houver alterações na organização, na legislação ou nas partes interessadas, a tabela deve ser revista e atualizada.</t>
+  </si>
+  <si>
+    <t>Sempre que possível, associe as necessidades identificadas aos riscos, oportunidades e ações previstas no Sistema de Gestão.</t>
+  </si>
+  <si>
+    <t>GUIA DE PREENCHIMENTO</t>
+  </si>
+  <si>
+    <t>Em palavras simples:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A ISO não exige apenas que a organização faça uma tabela com as partes interessadas. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ela quer que fique claro por que essa análise existe e como ela é utilizada. 
+</t>
+  </si>
+  <si>
+    <t>Esse pequeno texto funciona como uma introdução ao documento e demonstra que a organização compreende o objetivo do requisito 4.2.</t>
+  </si>
+  <si>
+    <t>EXPLICAÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">identificar as partes interessadas, entender o que elas esperam e verificar quais dessas expectativas </t>
+  </si>
+  <si>
+    <t>que precisam ser cumpridas pelo Sistema de Gestão.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ela deve ser revista periodicamente ou sempre que houver mudanças importantes, como alteração de legislação, </t>
+  </si>
+  <si>
+    <t>novos clientes, novos fornecedores ou mudanças na própria organização. Isso demonstra que o SGI está atualizado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O primeiro parágrafo explica o que este documento faz: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">O segundo parágrafo explica por que isso é importante: </t>
+  </si>
+  <si>
+    <t>O último parágrafo mostra que esta análise não é um documento feito uma única vez:</t>
+  </si>
+  <si>
+    <t>entre outros, consegue tomar melhores decisões, evitar problemas, cumprir a legislação e melhorar continuamente.</t>
+  </si>
+  <si>
+    <t>quando a empresa conhece as expectativas dos clientes, trabalhadores, fornecedores, entidades reguladoras,</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,6 +331,47 @@
       <name val="Cambria"/>
       <family val="1"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="0"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="0"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="26"/>
+      <color theme="0"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -163,7 +393,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -199,11 +429,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -227,6 +483,34 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -235,8 +519,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF203E5E"/>
       <color rgb="FF0F7343"/>
-      <color rgb="FF203E5E"/>
     </mruColors>
   </colors>
   <extLst>
@@ -254,16 +538,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>53340</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1127760</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>677037</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -293,8 +577,120 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="289560" y="0"/>
-          <a:ext cx="1074420" cy="1066800"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="913257" cy="906780"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>791337</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7DDA751A-1E33-4E6A-BACB-E43DDC4FC9D0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="9143" t="9714" r="10285" b="10285"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="913257" cy="906780"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>899160</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>153426</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagem 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B02CDB70-A9F8-4043-AD21-CDA38DD0B4E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="9143" t="9714" r="10285" b="10285"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="83820" y="0"/>
+          <a:ext cx="929640" cy="923046"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -622,8 +1018,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{149C4A48-AD68-4C67-A92C-BCC1E9F4A378}">
-  <dimension ref="B1:F26"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{149C4A48-AD68-4C67-A92C-BCC1E9F4A378}">
+  <dimension ref="B1:F25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.44140625" customWidth="1"/>
@@ -640,10 +1036,10 @@
       <c r="D1" s="5"/>
     </row>
     <row r="2" spans="2:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="5"/>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="8" t="s">
         <v>21</v>
       </c>
+      <c r="C2" s="8"/>
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
       <c r="F2" s="8"/>
@@ -654,90 +1050,93 @@
       <c r="D3" s="5"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="5"/>
+      <c r="B4" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="4" t="s">
-        <v>15</v>
-      </c>
+    <row r="7" spans="2:6" ht="7.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="4"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
     </row>
-    <row r="8" spans="2:6" ht="7.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="4"/>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="4" t="s">
-        <v>18</v>
-      </c>
+    <row r="11" spans="2:6" ht="9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="4"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
     </row>
-    <row r="12" spans="2:6" ht="9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="4"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="4" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="6" t="s">
+      <c r="B13" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="2:6" ht="5.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="2:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="7" t="s">
+    <row r="14" spans="2:6" ht="5.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="2:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C15" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D15" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E15" s="7" t="s">
         <v>3</v>
       </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="2"/>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -745,7 +1144,7 @@
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -753,39 +1152,39 @@
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="2"/>
+      <c r="E19" s="1"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B20" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B21" s="3" t="s">
+      <c r="B20" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" ht="41.4" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -793,31 +1192,23 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B26" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="2"/>
-    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C2:F2"/>
+    <mergeCell ref="B2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -825,5 +1216,229 @@
     <oddFooter>&amp;L&amp;"Cambria,Normal"4.2 -  Matriz das Partes Interessadas&amp;C&amp;"Cambria,Negrito"&amp;P &amp;"Cambria,Normal"de &amp;"Cambria,Negrito"&amp;N&amp;R&amp;"Cambria,Normal"R0 - data</oddFooter>
   </headerFooter>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FDC5B5D-48A1-4C81-B425-3D04A7DD6CF6}">
+  <dimension ref="B2:N15"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="1.77734375" style="12" customWidth="1"/>
+    <col min="2" max="2" width="50.109375" style="12" customWidth="1"/>
+    <col min="3" max="3" width="102.77734375" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="12"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:14" ht="55.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B4" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B5" s="12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" ht="8.4" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B8" s="12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" ht="4.8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="2:14" ht="19.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B11" s="14"/>
+      <c r="C11" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+    </row>
+    <row r="12" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+    </row>
+    <row r="13" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="19"/>
+      <c r="C13" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B14" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B15" s="14"/>
+      <c r="C15" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B12:B13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{348A956E-EBFA-43EA-87FD-CF8ECE13BBCA}">
+  <dimension ref="B2:F9"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="1.6640625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="25.44140625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="42.77734375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="41.33203125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="2.21875" style="4" customWidth="1"/>
+    <col min="6" max="6" width="51" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+    </row>
+    <row r="4" spans="2:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="55.2" x14ac:dyDescent="0.25">
+      <c r="B5" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="82.8" x14ac:dyDescent="0.25">
+      <c r="B6" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="69" x14ac:dyDescent="0.25">
+      <c r="B7" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="82.8" x14ac:dyDescent="0.25">
+      <c r="B8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="F9" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>